<commit_message>
update the graphs and insights
</commit_message>
<xml_diff>
--- a/results/performance_comparison.xlsx
+++ b/results/performance_comparison.xlsx
@@ -310,7 +310,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>CPython pyperformance — Surface Laptop 15 (X Plus)</a:t>
+              <a:t>CPython pyperformance — Surface Laptop 15 (X Elite)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -2429,9 +2429,9 @@
     <col width="39" customWidth="1" min="3" max="3"/>
     <col width="39" customWidth="1" min="4" max="4"/>
     <col width="41" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="37" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2465,19 +2465,19 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)
+          <t>Surface Laptop 15 (X Elite)
 LLVM</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)
+          <t>Surface Laptop 15 (X Elite)
 MSVC</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)
+          <t>Surface Laptop 15 (X Elite)
 Δ LLVM</t>
         </is>
       </c>
@@ -2634,7 +2634,7 @@
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)</t>
+          <t>Surface Laptop 15 (X Elite)</t>
         </is>
       </c>
     </row>
@@ -2793,7 +2793,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus) — LLVM</t>
+          <t>Surface Laptop 15 (X Elite) — LLVM</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -2812,7 +2812,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus) — MSVC</t>
+          <t>Surface Laptop 15 (X Elite) — MSVC</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -2845,7 +2845,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)</t>
+          <t>Surface Laptop 15 (X Elite)</t>
         </is>
       </c>
     </row>
@@ -2981,7 +2981,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)</t>
+          <t>Surface Laptop 15 (X Elite)</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -3060,7 +3060,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)</t>
+          <t>Surface Laptop 15 (X Elite)</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -3196,7 +3196,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)</t>
+          <t>Surface Laptop 15 (X Elite)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3219,7 +3219,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)</t>
+          <t>Surface Laptop 15 (X Elite)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3242,7 +3242,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)</t>
+          <t>Surface Laptop 15 (X Elite)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3988,7 +3988,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)</t>
+          <t>Surface Laptop 15 (X Elite)</t>
         </is>
       </c>
       <c r="B3" t="n">

</xml_diff>

<commit_message>
re-bench surface with latest msvc
</commit_message>
<xml_diff>
--- a/results/performance_comparison.xlsx
+++ b/results/performance_comparison.xlsx
@@ -310,7 +310,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>CPython pyperformance — Surface Laptop 15 (X Plus)</a:t>
+              <a:t>CPython pyperformance — Surface Laptop 15 (X Elite)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -2429,9 +2429,9 @@
     <col width="39" customWidth="1" min="3" max="3"/>
     <col width="39" customWidth="1" min="4" max="4"/>
     <col width="41" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="37" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2465,19 +2465,19 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)
+          <t>Surface Laptop 15 (X Elite)
 LLVM</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)
+          <t>Surface Laptop 15 (X Elite)
 MSVC</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)
+          <t>Surface Laptop 15 (X Elite)
 Δ LLVM</t>
         </is>
       </c>
@@ -2505,14 +2505,14 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.4017</v>
+        <v>0.4019</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5762</v>
+        <v>0.5987</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>+30.3%</t>
+          <t>+32.9%</t>
         </is>
       </c>
     </row>
@@ -2539,14 +2539,14 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>9.84</v>
+        <v>10.02</v>
       </c>
       <c r="G3" t="n">
-        <v>7.7</v>
+        <v>7.74</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>+27.7%</t>
+          <t>+29.4%</t>
         </is>
       </c>
     </row>
@@ -2573,14 +2573,14 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>7.4396</v>
+        <v>7.3779</v>
       </c>
       <c r="G4" t="n">
-        <v>13.0602</v>
+        <v>13.1347</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>+43.0%</t>
+          <t>+43.8%</t>
         </is>
       </c>
     </row>
@@ -2596,25 +2596,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.05937</v>
+        <v>0.059291</v>
       </c>
       <c r="D5" t="n">
         <v>0.076072</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>+22.0%</t>
+          <t>+22.1%</t>
         </is>
       </c>
       <c r="F5" t="n">
         <v>0.032112</v>
       </c>
       <c r="G5" t="n">
-        <v>0.048782</v>
+        <v>0.049791</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>+34.2%</t>
+          <t>+35.5%</t>
         </is>
       </c>
     </row>
@@ -2634,7 +2634,7 @@
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)</t>
+          <t>Surface Laptop 15 (X Elite)</t>
         </is>
       </c>
     </row>
@@ -2664,7 +2664,7 @@
         <v>1.4</v>
       </c>
       <c r="C2" t="n">
-        <v>1.43</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="3">
@@ -2677,7 +2677,7 @@
         <v>1.3</v>
       </c>
       <c r="C3" t="n">
-        <v>1.28</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="4">
@@ -2690,7 +2690,7 @@
         <v>1.15</v>
       </c>
       <c r="C4" t="n">
-        <v>1.76</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="5">
@@ -2703,7 +2703,7 @@
         <v>1.28</v>
       </c>
       <c r="C5" t="n">
-        <v>1.52</v>
+        <v>1.55</v>
       </c>
     </row>
   </sheetData>
@@ -2768,7 +2768,7 @@
         <v>23.44</v>
       </c>
       <c r="E2" t="n">
-        <v>16.84</v>
+        <v>16.87</v>
       </c>
     </row>
     <row r="3">
@@ -2793,17 +2793,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus) — LLVM</t>
+          <t>Surface Laptop 15 (X Elite) — LLVM</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2.489</v>
+        <v>2.488</v>
       </c>
       <c r="C4" t="n">
-        <v>9.84</v>
+        <v>10.02</v>
       </c>
       <c r="D4" t="n">
-        <v>38.77</v>
+        <v>38.82</v>
       </c>
       <c r="E4" t="n">
         <v>31.14</v>
@@ -2812,20 +2812,20 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus) — MSVC</t>
+          <t>Surface Laptop 15 (X Elite) — MSVC</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.735</v>
+        <v>1.67</v>
       </c>
       <c r="C5" t="n">
-        <v>7.7</v>
+        <v>7.74</v>
       </c>
       <c r="D5" t="n">
-        <v>15.63</v>
+        <v>15.83</v>
       </c>
       <c r="E5" t="n">
-        <v>20.5</v>
+        <v>20.08</v>
       </c>
     </row>
   </sheetData>
@@ -2845,7 +2845,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)</t>
+          <t>Surface Laptop 15 (X Elite)</t>
         </is>
       </c>
     </row>
@@ -2875,7 +2875,7 @@
         <v>28.6</v>
       </c>
       <c r="C2" t="n">
-        <v>30.3</v>
+        <v>32.9</v>
       </c>
     </row>
     <row r="3">
@@ -2888,7 +2888,7 @@
         <v>29.7</v>
       </c>
       <c r="C3" t="n">
-        <v>27.7</v>
+        <v>29.4</v>
       </c>
     </row>
     <row r="4">
@@ -2901,7 +2901,7 @@
         <v>13</v>
       </c>
       <c r="C4" t="n">
-        <v>43</v>
+        <v>43.8</v>
       </c>
     </row>
     <row r="5">
@@ -2911,10 +2911,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>22</v>
+        <v>22.1</v>
       </c>
       <c r="C5" t="n">
-        <v>34.2</v>
+        <v>35.5</v>
       </c>
     </row>
   </sheetData>
@@ -2981,18 +2981,18 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)</t>
+          <t>Surface Laptop 15 (X Elite)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.4017</v>
+        <v>0.4019</v>
       </c>
       <c r="C3" t="n">
-        <v>0.5762</v>
+        <v>0.5987</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>+30.3%</t>
+          <t>+32.9%</t>
         </is>
       </c>
     </row>
@@ -3060,18 +3060,18 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)</t>
+          <t>Surface Laptop 15 (X Elite)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>9.84</v>
+        <v>10.02</v>
       </c>
       <c r="C3" t="n">
-        <v>7.7</v>
+        <v>7.74</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>+27.7%</t>
+          <t>+29.4%</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)</t>
+          <t>Surface Laptop 15 (X Elite)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3205,21 +3205,21 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2.146</v>
+        <v>2.1133</v>
       </c>
       <c r="D5" t="n">
-        <v>2.6668</v>
+        <v>2.7306</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>+19.5%</t>
+          <t>+22.6%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)</t>
+          <t>Surface Laptop 15 (X Elite)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3228,21 +3228,21 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>25.7914</v>
+        <v>25.7575</v>
       </c>
       <c r="D6" t="n">
-        <v>63.9603</v>
+        <v>63.1817</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>+59.7%</t>
+          <t>+59.2%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)</t>
+          <t>Surface Laptop 15 (X Elite)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3251,14 +3251,14 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>7.4396</v>
+        <v>7.3779</v>
       </c>
       <c r="D7" t="n">
-        <v>13.0602</v>
+        <v>13.1347</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>+43.0%</t>
+          <t>+43.8%</t>
         </is>
       </c>
     </row>
@@ -3312,14 +3312,14 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.095346</v>
+        <v>0.095429</v>
       </c>
       <c r="C2" t="n">
         <v>0.124772</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>+23.6%</t>
+          <t>+23.5%</t>
         </is>
       </c>
     </row>
@@ -3330,14 +3330,14 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.130121</v>
+        <v>0.129962</v>
       </c>
       <c r="C3" t="n">
         <v>0.158947</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>+18.1%</t>
+          <t>+18.2%</t>
         </is>
       </c>
     </row>
@@ -3348,7 +3348,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.005373</v>
+        <v>0.005367</v>
       </c>
       <c r="C4" t="n">
         <v>0.007628</v>
@@ -3366,14 +3366,14 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.663334</v>
+        <v>0.6640779999999999</v>
       </c>
       <c r="C5" t="n">
         <v>0.797839</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>+16.9%</t>
+          <t>+16.8%</t>
         </is>
       </c>
     </row>
@@ -3384,14 +3384,14 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.112637</v>
+        <v>0.112435</v>
       </c>
       <c r="C6" t="n">
         <v>0.14388</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>+21.7%</t>
+          <t>+21.9%</t>
         </is>
       </c>
     </row>
@@ -3402,7 +3402,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.169239</v>
+        <v>0.16925</v>
       </c>
       <c r="C7" t="n">
         <v>0.238859</v>
@@ -3420,14 +3420,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.009993</v>
+        <v>0.010005</v>
       </c>
       <c r="C8" t="n">
         <v>0.013346</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>+25.1%</t>
+          <t>+25.0%</t>
         </is>
       </c>
     </row>
@@ -3438,14 +3438,14 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.165362</v>
+        <v>0.165475</v>
       </c>
       <c r="C9" t="n">
         <v>0.216421</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>+23.6%</t>
+          <t>+23.5%</t>
         </is>
       </c>
     </row>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>+26.9%</t>
+          <t>+27.0%</t>
         </is>
       </c>
     </row>
@@ -3474,14 +3474,14 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.327896</v>
+        <v>0.326568</v>
       </c>
       <c r="C11" t="n">
         <v>0.310823</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-5.5%</t>
+          <t>-5.1%</t>
         </is>
       </c>
     </row>
@@ -3492,7 +3492,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.72216</v>
+        <v>0.722034</v>
       </c>
       <c r="C12" t="n">
         <v>0.905057</v>
@@ -3510,7 +3510,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.437276</v>
+        <v>0.437358</v>
       </c>
       <c r="C13" t="n">
         <v>0.576114</v>
@@ -3528,14 +3528,14 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.068816</v>
+        <v>0.068924</v>
       </c>
       <c r="C14" t="n">
         <v>0.098366</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>+30.0%</t>
+          <t>+29.9%</t>
         </is>
       </c>
     </row>
@@ -3546,14 +3546,14 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.181833</v>
+        <v>0.178376</v>
       </c>
       <c r="C15" t="n">
         <v>0.216284</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>+15.9%</t>
+          <t>+17.5%</t>
         </is>
       </c>
     </row>
@@ -3564,14 +3564,14 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.000395</v>
+        <v>0.000396</v>
       </c>
       <c r="C16" t="n">
         <v>0.000519</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>+24.0%</t>
+          <t>+23.8%</t>
         </is>
       </c>
     </row>
@@ -3582,14 +3582,14 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.05937</v>
+        <v>0.059291</v>
       </c>
       <c r="C17" t="n">
         <v>0.076072</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>+22.0%</t>
+          <t>+22.1%</t>
         </is>
       </c>
     </row>
@@ -3646,11 +3646,11 @@
         <v>0.048154</v>
       </c>
       <c r="C2" t="n">
-        <v>0.08004</v>
+        <v>0.080566</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>+39.8%</t>
+          <t>+40.2%</t>
         </is>
       </c>
     </row>
@@ -3664,11 +3664,11 @@
         <v>0.063358</v>
       </c>
       <c r="C3" t="n">
-        <v>0.097455</v>
+        <v>0.09900299999999999</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>+35.0%</t>
+          <t>+36.0%</t>
         </is>
       </c>
     </row>
@@ -3682,11 +3682,11 @@
         <v>0.003084</v>
       </c>
       <c r="C4" t="n">
-        <v>0.005397</v>
+        <v>0.00543</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>+42.9%</t>
+          <t>+43.2%</t>
         </is>
       </c>
     </row>
@@ -3700,11 +3700,11 @@
         <v>0.354055</v>
       </c>
       <c r="C5" t="n">
-        <v>0.478173</v>
+        <v>0.48759</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>+26.0%</t>
+          <t>+27.4%</t>
         </is>
       </c>
     </row>
@@ -3718,11 +3718,11 @@
         <v>0.063611</v>
       </c>
       <c r="C6" t="n">
-        <v>0.09370299999999999</v>
+        <v>0.09683600000000001</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>+32.1%</t>
+          <t>+34.3%</t>
         </is>
       </c>
     </row>
@@ -3736,11 +3736,11 @@
         <v>0.100693</v>
       </c>
       <c r="C7" t="n">
-        <v>0.171437</v>
+        <v>0.179047</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>+41.3%</t>
+          <t>+43.8%</t>
         </is>
       </c>
     </row>
@@ -3754,11 +3754,11 @@
         <v>0.005527</v>
       </c>
       <c r="C8" t="n">
-        <v>0.009055000000000001</v>
+        <v>0.009919000000000001</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>+39.0%</t>
+          <t>+44.3%</t>
         </is>
       </c>
     </row>
@@ -3772,11 +3772,11 @@
         <v>0.09575699999999999</v>
       </c>
       <c r="C9" t="n">
-        <v>0.131222</v>
+        <v>0.136929</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>+27.0%</t>
+          <t>+30.1%</t>
         </is>
       </c>
     </row>
@@ -3790,11 +3790,11 @@
         <v>0.000256</v>
       </c>
       <c r="C10" t="n">
-        <v>0.00043</v>
+        <v>0.000435</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>+40.6%</t>
+          <t>+41.2%</t>
         </is>
       </c>
     </row>
@@ -3808,11 +3808,11 @@
         <v>0.249397</v>
       </c>
       <c r="C11" t="n">
-        <v>0.20094</v>
+        <v>0.197559</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-24.1%</t>
+          <t>-26.2%</t>
         </is>
       </c>
     </row>
@@ -3826,11 +3826,11 @@
         <v>0.391455</v>
       </c>
       <c r="C12" t="n">
-        <v>0.581027</v>
+        <v>0.590601</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>+32.6%</t>
+          <t>+33.7%</t>
         </is>
       </c>
     </row>
@@ -3844,11 +3844,11 @@
         <v>0.214372</v>
       </c>
       <c r="C13" t="n">
-        <v>0.354376</v>
+        <v>0.357957</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>+39.5%</t>
+          <t>+40.1%</t>
         </is>
       </c>
     </row>
@@ -3862,11 +3862,11 @@
         <v>0.040384</v>
       </c>
       <c r="C14" t="n">
-        <v>0.065813</v>
+        <v>0.066819</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>+38.6%</t>
+          <t>+39.6%</t>
         </is>
       </c>
     </row>
@@ -3880,11 +3880,11 @@
         <v>0.08543100000000001</v>
       </c>
       <c r="C15" t="n">
-        <v>0.141301</v>
+        <v>0.142996</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>+39.5%</t>
+          <t>+40.3%</t>
         </is>
       </c>
     </row>
@@ -3898,11 +3898,11 @@
         <v>0.000191</v>
       </c>
       <c r="C16" t="n">
-        <v>0.000331</v>
+        <v>0.000332</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>+42.4%</t>
+          <t>+42.5%</t>
         </is>
       </c>
     </row>
@@ -3916,11 +3916,11 @@
         <v>0.032112</v>
       </c>
       <c r="C17" t="n">
-        <v>0.048782</v>
+        <v>0.049791</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>+34.2%</t>
+          <t>+35.5%</t>
         </is>
       </c>
     </row>
@@ -3974,32 +3974,32 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.05937</v>
+        <v>0.059291</v>
       </c>
       <c r="C2" t="n">
         <v>0.076072</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>+22.0%</t>
+          <t>+22.1%</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Surface Laptop 15 (X Plus)</t>
+          <t>Surface Laptop 15 (X Elite)</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>0.032112</v>
       </c>
       <c r="C3" t="n">
-        <v>0.048782</v>
+        <v>0.049791</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>+34.2%</t>
+          <t>+35.5%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
re-bench volterra with 14.51
</commit_message>
<xml_diff>
--- a/results/performance_comparison.xlsx
+++ b/results/performance_comparison.xlsx
@@ -2497,11 +2497,11 @@
         <v>0.8101</v>
       </c>
       <c r="D2" t="n">
-        <v>1.1352</v>
+        <v>1.1435</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>+28.6%</t>
+          <t>+29.1%</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -2528,14 +2528,14 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4.51</v>
+        <v>4.48</v>
       </c>
       <c r="D3" t="n">
-        <v>3.48</v>
+        <v>3.74</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>+29.7%</t>
+          <t>+19.6%</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -2565,11 +2565,11 @@
         <v>13.3992</v>
       </c>
       <c r="D4" t="n">
-        <v>15.3968</v>
+        <v>18.8578</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>+13.0%</t>
+          <t>+28.9%</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -2599,11 +2599,11 @@
         <v>0.059291</v>
       </c>
       <c r="D5" t="n">
-        <v>0.076072</v>
+        <v>0.076322</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>+22.1%</t>
+          <t>+22.3%</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -2661,7 +2661,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.4</v>
+        <v>1.41</v>
       </c>
       <c r="C2" t="n">
         <v>1.49</v>
@@ -2674,7 +2674,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="C3" t="n">
         <v>1.29</v>
@@ -2687,7 +2687,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.15</v>
+        <v>1.41</v>
       </c>
       <c r="C4" t="n">
         <v>1.78</v>
@@ -2700,7 +2700,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.28</v>
+        <v>1.29</v>
       </c>
       <c r="C5" t="n">
         <v>1.55</v>
@@ -2762,7 +2762,7 @@
         <v>1.234</v>
       </c>
       <c r="C2" t="n">
-        <v>4.51</v>
+        <v>4.48</v>
       </c>
       <c r="D2" t="n">
         <v>23.44</v>
@@ -2778,16 +2778,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.881</v>
+        <v>0.875</v>
       </c>
       <c r="C3" t="n">
-        <v>3.48</v>
+        <v>3.74</v>
       </c>
       <c r="D3" t="n">
-        <v>12.38</v>
+        <v>12.15</v>
       </c>
       <c r="E3" t="n">
-        <v>13.15</v>
+        <v>13.1</v>
       </c>
     </row>
     <row r="4">
@@ -2872,7 +2872,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>28.6</v>
+        <v>29.1</v>
       </c>
       <c r="C2" t="n">
         <v>32.9</v>
@@ -2885,7 +2885,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>29.7</v>
+        <v>19.6</v>
       </c>
       <c r="C3" t="n">
         <v>29.4</v>
@@ -2898,7 +2898,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>13</v>
+        <v>28.9</v>
       </c>
       <c r="C4" t="n">
         <v>43.8</v>
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>22.1</v>
+        <v>22.3</v>
       </c>
       <c r="C5" t="n">
         <v>35.5</v>
@@ -2970,11 +2970,11 @@
         <v>0.8101</v>
       </c>
       <c r="C2" t="n">
-        <v>1.1352</v>
+        <v>1.1435</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>+28.6%</t>
+          <t>+29.1%</t>
         </is>
       </c>
     </row>
@@ -3046,14 +3046,14 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4.51</v>
+        <v>4.48</v>
       </c>
       <c r="C2" t="n">
-        <v>3.48</v>
+        <v>3.74</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>+29.7%</t>
+          <t>+19.6%</t>
         </is>
       </c>
     </row>
@@ -3139,11 +3139,11 @@
         <v>4.2088</v>
       </c>
       <c r="D2" t="n">
-        <v>2.9355</v>
+        <v>4.3221</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>-43.4%</t>
+          <t>+2.6%</t>
         </is>
       </c>
     </row>
@@ -3162,11 +3162,11 @@
         <v>42.6579</v>
       </c>
       <c r="D3" t="n">
-        <v>80.75539999999999</v>
+        <v>82.2784</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>+47.2%</t>
+          <t>+48.2%</t>
         </is>
       </c>
     </row>
@@ -3185,11 +3185,11 @@
         <v>13.3992</v>
       </c>
       <c r="D4" t="n">
-        <v>15.3968</v>
+        <v>18.8578</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>+13.0%</t>
+          <t>+28.9%</t>
         </is>
       </c>
     </row>
@@ -3315,11 +3315,11 @@
         <v>0.095429</v>
       </c>
       <c r="C2" t="n">
-        <v>0.124772</v>
+        <v>0.125281</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>+23.5%</t>
+          <t>+23.8%</t>
         </is>
       </c>
     </row>
@@ -3333,11 +3333,11 @@
         <v>0.129962</v>
       </c>
       <c r="C3" t="n">
-        <v>0.158947</v>
+        <v>0.159653</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>+18.2%</t>
+          <t>+18.6%</t>
         </is>
       </c>
     </row>
@@ -3351,11 +3351,11 @@
         <v>0.005367</v>
       </c>
       <c r="C4" t="n">
-        <v>0.007628</v>
+        <v>0.00765</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>+29.6%</t>
+          <t>+29.8%</t>
         </is>
       </c>
     </row>
@@ -3369,11 +3369,11 @@
         <v>0.6640779999999999</v>
       </c>
       <c r="C5" t="n">
-        <v>0.797839</v>
+        <v>0.799219</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>+16.8%</t>
+          <t>+16.9%</t>
         </is>
       </c>
     </row>
@@ -3387,11 +3387,11 @@
         <v>0.112435</v>
       </c>
       <c r="C6" t="n">
-        <v>0.14388</v>
+        <v>0.143855</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>+21.9%</t>
+          <t>+21.8%</t>
         </is>
       </c>
     </row>
@@ -3405,11 +3405,11 @@
         <v>0.16925</v>
       </c>
       <c r="C7" t="n">
-        <v>0.238859</v>
+        <v>0.23954</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>+29.1%</t>
+          <t>+29.3%</t>
         </is>
       </c>
     </row>
@@ -3423,11 +3423,11 @@
         <v>0.010005</v>
       </c>
       <c r="C8" t="n">
-        <v>0.013346</v>
+        <v>0.013383</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>+25.0%</t>
+          <t>+25.2%</t>
         </is>
       </c>
     </row>
@@ -3441,11 +3441,11 @@
         <v>0.165475</v>
       </c>
       <c r="C9" t="n">
-        <v>0.216421</v>
+        <v>0.217375</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>+23.5%</t>
+          <t>+23.9%</t>
         </is>
       </c>
     </row>
@@ -3459,11 +3459,11 @@
         <v>0.000563</v>
       </c>
       <c r="C10" t="n">
-        <v>0.000771</v>
+        <v>0.000777</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>+27.0%</t>
+          <t>+27.5%</t>
         </is>
       </c>
     </row>
@@ -3477,11 +3477,11 @@
         <v>0.326568</v>
       </c>
       <c r="C11" t="n">
-        <v>0.310823</v>
+        <v>0.311463</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-5.1%</t>
+          <t>-4.8%</t>
         </is>
       </c>
     </row>
@@ -3495,11 +3495,11 @@
         <v>0.722034</v>
       </c>
       <c r="C12" t="n">
-        <v>0.905057</v>
+        <v>0.909702</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>+20.2%</t>
+          <t>+20.6%</t>
         </is>
       </c>
     </row>
@@ -3513,11 +3513,11 @@
         <v>0.437358</v>
       </c>
       <c r="C13" t="n">
-        <v>0.576114</v>
+        <v>0.578641</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>+24.1%</t>
+          <t>+24.4%</t>
         </is>
       </c>
     </row>
@@ -3531,11 +3531,11 @@
         <v>0.068924</v>
       </c>
       <c r="C14" t="n">
-        <v>0.098366</v>
+        <v>0.09858</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>+29.9%</t>
+          <t>+30.1%</t>
         </is>
       </c>
     </row>
@@ -3549,7 +3549,7 @@
         <v>0.178376</v>
       </c>
       <c r="C15" t="n">
-        <v>0.216284</v>
+        <v>0.216095</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -3567,11 +3567,11 @@
         <v>0.000396</v>
       </c>
       <c r="C16" t="n">
-        <v>0.000519</v>
+        <v>0.000522</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>+23.8%</t>
+          <t>+24.2%</t>
         </is>
       </c>
     </row>
@@ -3585,11 +3585,11 @@
         <v>0.059291</v>
       </c>
       <c r="C17" t="n">
-        <v>0.076072</v>
+        <v>0.076322</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>+22.1%</t>
+          <t>+22.3%</t>
         </is>
       </c>
     </row>
@@ -3977,11 +3977,11 @@
         <v>0.059291</v>
       </c>
       <c r="C2" t="n">
-        <v>0.076072</v>
+        <v>0.076322</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>+22.1%</t>
+          <t>+22.3%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix 14.51 usage for cpython and lame, update insights
</commit_message>
<xml_diff>
--- a/results/performance_comparison.xlsx
+++ b/results/performance_comparison.xlsx
@@ -2497,11 +2497,11 @@
         <v>0.8101</v>
       </c>
       <c r="D2" t="n">
-        <v>1.1435</v>
+        <v>1.1044</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>+29.1%</t>
+          <t>+26.6%</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -2599,11 +2599,11 @@
         <v>0.059291</v>
       </c>
       <c r="D5" t="n">
-        <v>0.076322</v>
+        <v>0.078197</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>+22.3%</t>
+          <t>+24.2%</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -2661,7 +2661,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.41</v>
+        <v>1.36</v>
       </c>
       <c r="C2" t="n">
         <v>1.49</v>
@@ -2700,7 +2700,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.29</v>
+        <v>1.32</v>
       </c>
       <c r="C5" t="n">
         <v>1.55</v>
@@ -2778,7 +2778,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.875</v>
+        <v>0.905</v>
       </c>
       <c r="C3" t="n">
         <v>3.74</v>
@@ -2787,7 +2787,7 @@
         <v>12.15</v>
       </c>
       <c r="E3" t="n">
-        <v>13.1</v>
+        <v>12.79</v>
       </c>
     </row>
     <row r="4">
@@ -2872,7 +2872,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>29.1</v>
+        <v>26.6</v>
       </c>
       <c r="C2" t="n">
         <v>32.9</v>
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>22.3</v>
+        <v>24.2</v>
       </c>
       <c r="C5" t="n">
         <v>35.5</v>
@@ -2970,11 +2970,11 @@
         <v>0.8101</v>
       </c>
       <c r="C2" t="n">
-        <v>1.1435</v>
+        <v>1.1044</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>+29.1%</t>
+          <t>+26.6%</t>
         </is>
       </c>
     </row>
@@ -3315,11 +3315,11 @@
         <v>0.095429</v>
       </c>
       <c r="C2" t="n">
-        <v>0.125281</v>
+        <v>0.128839</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>+23.8%</t>
+          <t>+25.9%</t>
         </is>
       </c>
     </row>
@@ -3333,11 +3333,11 @@
         <v>0.129962</v>
       </c>
       <c r="C3" t="n">
-        <v>0.159653</v>
+        <v>0.160039</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>+18.6%</t>
+          <t>+18.8%</t>
         </is>
       </c>
     </row>
@@ -3351,11 +3351,11 @@
         <v>0.005367</v>
       </c>
       <c r="C4" t="n">
-        <v>0.00765</v>
+        <v>0.007816</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>+29.8%</t>
+          <t>+31.3%</t>
         </is>
       </c>
     </row>
@@ -3369,11 +3369,11 @@
         <v>0.6640779999999999</v>
       </c>
       <c r="C5" t="n">
-        <v>0.799219</v>
+        <v>0.823371</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>+16.9%</t>
+          <t>+19.3%</t>
         </is>
       </c>
     </row>
@@ -3387,11 +3387,11 @@
         <v>0.112435</v>
       </c>
       <c r="C6" t="n">
-        <v>0.143855</v>
+        <v>0.147175</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>+21.8%</t>
+          <t>+23.6%</t>
         </is>
       </c>
     </row>
@@ -3405,11 +3405,11 @@
         <v>0.16925</v>
       </c>
       <c r="C7" t="n">
-        <v>0.23954</v>
+        <v>0.247973</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>+29.3%</t>
+          <t>+31.7%</t>
         </is>
       </c>
     </row>
@@ -3423,11 +3423,11 @@
         <v>0.010005</v>
       </c>
       <c r="C8" t="n">
-        <v>0.013383</v>
+        <v>0.013914</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>+25.2%</t>
+          <t>+28.1%</t>
         </is>
       </c>
     </row>
@@ -3441,11 +3441,11 @@
         <v>0.165475</v>
       </c>
       <c r="C9" t="n">
-        <v>0.217375</v>
+        <v>0.218884</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>+23.9%</t>
+          <t>+24.4%</t>
         </is>
       </c>
     </row>
@@ -3459,11 +3459,11 @@
         <v>0.000563</v>
       </c>
       <c r="C10" t="n">
-        <v>0.000777</v>
+        <v>0.000764</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>+27.5%</t>
+          <t>+26.3%</t>
         </is>
       </c>
     </row>
@@ -3477,11 +3477,11 @@
         <v>0.326568</v>
       </c>
       <c r="C11" t="n">
-        <v>0.311463</v>
+        <v>0.319713</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-4.8%</t>
+          <t>-2.1%</t>
         </is>
       </c>
     </row>
@@ -3495,11 +3495,11 @@
         <v>0.722034</v>
       </c>
       <c r="C12" t="n">
-        <v>0.909702</v>
+        <v>0.939729</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>+20.6%</t>
+          <t>+23.2%</t>
         </is>
       </c>
     </row>
@@ -3513,11 +3513,11 @@
         <v>0.437358</v>
       </c>
       <c r="C13" t="n">
-        <v>0.578641</v>
+        <v>0.600599</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>+24.4%</t>
+          <t>+27.2%</t>
         </is>
       </c>
     </row>
@@ -3531,11 +3531,11 @@
         <v>0.068924</v>
       </c>
       <c r="C14" t="n">
-        <v>0.09858</v>
+        <v>0.09783600000000001</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>+30.1%</t>
+          <t>+29.6%</t>
         </is>
       </c>
     </row>
@@ -3549,11 +3549,11 @@
         <v>0.178376</v>
       </c>
       <c r="C15" t="n">
-        <v>0.216095</v>
+        <v>0.227507</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>+17.5%</t>
+          <t>+21.6%</t>
         </is>
       </c>
     </row>
@@ -3567,11 +3567,11 @@
         <v>0.000396</v>
       </c>
       <c r="C16" t="n">
-        <v>0.000522</v>
+        <v>0.000552</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>+24.2%</t>
+          <t>+28.3%</t>
         </is>
       </c>
     </row>
@@ -3585,11 +3585,11 @@
         <v>0.059291</v>
       </c>
       <c r="C17" t="n">
-        <v>0.076322</v>
+        <v>0.078197</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>+22.3%</t>
+          <t>+24.2%</t>
         </is>
       </c>
     </row>
@@ -3977,11 +3977,11 @@
         <v>0.059291</v>
       </c>
       <c r="C2" t="n">
-        <v>0.076322</v>
+        <v>0.078197</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>+22.3%</t>
+          <t>+24.2%</t>
         </is>
       </c>
     </row>

</xml_diff>